<commit_message>
data: fix concept_additions (berry/Finnish+Greek clobbered by an off-by-one); rebuild NEL qc sheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/concept_additions.xlsx
+++ b/data/raw/concept_additions.xlsx
@@ -1155,9 +1155,14 @@
           <t>bogyó</t>
         </is>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>marja</t>
+        </is>
+      </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>marja</t>
+          <t>μούρο</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1277,7 +1282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1293,17 +1298,22 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>ours_google</t>
+          <t>ours</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>northeuralex_orth</t>
+          <t>northeuralex_orth (attested)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
           <t>verdict</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>note</t>
         </is>
       </c>
     </row>
@@ -1333,6 +1343,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1360,6 +1371,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1387,6 +1399,7 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1414,6 +1427,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1441,6 +1455,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1468,6 +1483,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1495,6 +1511,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1522,6 +1539,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1531,24 +1549,21 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Vietnamese</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>翼</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>羽</t>
-        </is>
-      </c>
+          <t>cánh</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1558,17 +1573,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>Japanese</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>비행</t>
+          <t>翼</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>날개</t>
+          <t>羽</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1576,6 +1591,7 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1585,24 +1601,25 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>Korean</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>kanat</t>
+          <t>비행</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>kanat</t>
+          <t>날개</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1612,24 +1629,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Hebrew</t>
+          <t>Thai</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>אֲגַף</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>כנף</t>
-        </is>
-      </c>
+          <t>ปีก</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1639,44 +1653,41 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Indonesian</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>विंग</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>डैना, पंख</t>
-        </is>
-      </c>
+          <t>sayap</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>navel</t>
+          <t>wing</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Hungarian</t>
+          <t>Turkish</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>köldök</t>
+          <t>kanat</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>köldök</t>
+          <t>kanat</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1684,53 +1695,51 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>navel</t>
+          <t>wing</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Finnish</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>napa</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>napa</t>
-        </is>
-      </c>
+          <t>الجناح</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>navel</t>
+          <t>wing</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Greek</t>
+          <t>Hebrew</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ομφαλός</t>
+          <t>אֲגַף</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>αφαλός</t>
+          <t>כנף</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1738,60 +1747,59 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>navel</t>
+          <t>wing</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Russian</t>
+          <t>Swahili</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>пупок</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>пупок</t>
-        </is>
-      </c>
+          <t>mrengo</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>navel</t>
+          <t>wing</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nabel</t>
+          <t>विंग</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Nabel</t>
+          <t>डैना, पंख</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1801,17 +1809,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>Hungarian</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ombligo</t>
+          <t>köldök</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ombligo</t>
+          <t>köldök</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1819,6 +1827,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1828,17 +1837,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>Finnish</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ombelico</t>
+          <t>napa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ombelico</t>
+          <t>napa</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1846,6 +1855,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1855,24 +1865,25 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Welsh</t>
+          <t>Greek</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>bogail</t>
+          <t>ομφαλός</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>bogail</t>
+          <t>αφαλός</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1882,17 +1893,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Russian</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>へそ</t>
+          <t>пупок</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>へそ</t>
+          <t>пупок</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1900,6 +1911,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1909,17 +1921,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>German</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>배꼽</t>
+          <t>Nabel</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>배꼽</t>
+          <t>Nabel</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1927,6 +1939,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1936,17 +1949,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>Spanish</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>göbek</t>
+          <t>ombligo</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>göbek</t>
+          <t>ombligo</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1954,6 +1967,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1963,24 +1977,25 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Hebrew</t>
+          <t>Italian</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>טַבּוּר</t>
+          <t>ombelico</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>טבור</t>
+          <t>ombelico</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1990,17 +2005,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Welsh</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>नाभि</t>
+          <t>bogail</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>ढोंढी, नाभि</t>
+          <t>bogail</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -2008,276 +2023,267 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Hungarian</t>
+          <t>Vietnamese</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>comb</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>comb</t>
-        </is>
-      </c>
+          <t>rốn</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Finnish</t>
+          <t>Japanese</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>reiteen</t>
+          <t>へそ</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>reisi</t>
+          <t>へそ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Greek</t>
+          <t>Korean</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>μήρος</t>
+          <t>배꼽</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>μηρός</t>
+          <t>배꼽</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Russian</t>
+          <t>Thai</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>бедро</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>бедро</t>
-        </is>
-      </c>
+          <t>สะดือ</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Indonesian</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Oberschenkel</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Oberschenkel</t>
-        </is>
-      </c>
+          <t>pusar</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>Turkish</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>hermético</t>
+          <t>göbek</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>muslo</t>
+          <t>göbek</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>coscia</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>fèmore</t>
-        </is>
-      </c>
+          <t>سرة</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Welsh</t>
+          <t>Hebrew</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>clun</t>
+          <t>טַבּוּר</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>clun</t>
+          <t>טבור</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Swahili</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>大腿</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>上腿</t>
-        </is>
-      </c>
+          <t>kitovu</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>thigh</t>
+          <t>navel</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>대퇴골</t>
+          <t>नाभि</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>허벅다리</t>
+          <t>ढोंढी, नाभि</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2287,17 +2293,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>Hungarian</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>uyluk</t>
+          <t>comb</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>uyluk</t>
+          <t>comb</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -2305,6 +2311,7 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2314,17 +2321,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Hebrew</t>
+          <t>Finnish</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>יָרֵך</t>
+          <t>reiteen</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ירך</t>
+          <t>reisi</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -2332,6 +2339,7 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2341,17 +2349,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Greek</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>जाँघ</t>
+          <t>μήρος</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>उरु</t>
+          <t>μηρός</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -2359,53 +2367,55 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Hungarian</t>
+          <t>Russian</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>visz</t>
+          <t>бедро</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>hord</t>
+          <t>бедро</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Finnish</t>
+          <t>German</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>kantaa</t>
+          <t>Oberschenkel</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>kantaa</t>
+          <t>Oberschenkel</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2413,26 +2423,27 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Greek</t>
+          <t>Spanish</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>μεταφέρω</t>
+          <t>hermético</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>φέρνω</t>
+          <t>muslo</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2440,53 +2451,55 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Russian</t>
+          <t>Italian</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>нести</t>
+          <t>coscia</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>нести</t>
+          <t>fèmore</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Welsh</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>tragen</t>
+          <t>clun</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>tragen</t>
+          <t>clun</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2494,80 +2507,79 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>Vietnamese</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>llevar</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>llevar</t>
-        </is>
-      </c>
+          <t>đùi</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>Japanese</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>trasportare</t>
+          <t>大腿</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>portare</t>
+          <t>上腿</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Welsh</t>
+          <t>Korean</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>cario</t>
+          <t>대퇴골</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>cludo</t>
+          <t>허벅다리</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -2575,65 +2587,60 @@
           <t>DIFFER</t>
         </is>
       </c>
+      <c r="F48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Thai</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>運ぶ</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>運ぶ</t>
-        </is>
-      </c>
+          <t>ต้นขา</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>Indonesian</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>나르다</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>지우다</t>
-        </is>
-      </c>
+          <t>paha</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2643,12 +2650,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>taşımak</t>
+          <t>uyluk</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>taşımak</t>
+          <t>uyluk</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2656,523 +2663,587 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Hebrew</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>לשאת</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>נשא</t>
-        </is>
-      </c>
+          <t>فخذ</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>carry</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Hebrew</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ढोना</t>
+          <t>יָרֵך</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ढोना</t>
+          <t>ירך</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Hungarian</t>
+          <t>Swahili</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>darál</t>
-        </is>
-      </c>
+          <t>paja</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>no-ref</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>thigh</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Finnish</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>jauhaa</t>
+          <t>जाँघ</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>उरु</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Greek</t>
+          <t>Hungarian</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>αλέθω</t>
+          <t>visz</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>hord</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Russian</t>
+          <t>Finnish</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>молоть</t>
+          <t>kantaa</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>kantaa</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Greek</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>schleifen</t>
+          <t>μεταφέρω</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>φέρνω</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>Russian</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>moler</t>
+          <t>нести</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>нести</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>German</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>macinare</t>
+          <t>tragen</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>tragen</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Welsh</t>
+          <t>Spanish</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>malu</t>
+          <t>llevar</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>llevar</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Italian</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>粉砕する</t>
+          <t>trasportare</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>portare</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>Welsh</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>갈기</t>
+          <t>cario</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>cludo</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>Vietnamese</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>öğütmek</t>
-        </is>
-      </c>
+          <t>mang</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr">
         <is>
           <t>no-ref</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Hebrew</t>
+          <t>Japanese</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>לִטחוֹן</t>
+          <t>運ぶ</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>運ぶ</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>grind</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Korean</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>पिसना</t>
+          <t>나르다</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>지우다</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>no-ref</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Hungarian</t>
+          <t>Thai</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>bogyó</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>bogyó</t>
-        </is>
-      </c>
+          <t>พก</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Finnish</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>marja</t>
-        </is>
-      </c>
+          <t>Indonesian</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>membawa</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Greek</t>
+          <t>Turkish</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>μούρο</t>
+          <t>taşımak</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>ρόγα</t>
+          <t>taşımak</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Russian</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ягода</t>
-        </is>
-      </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>ягода</t>
-        </is>
-      </c>
+          <t>يحمل</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>German</t>
+          <t>Hebrew</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Beere</t>
+          <t>לשאת</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Beere</t>
+          <t>נשא</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Spanish</t>
+          <t>Swahili</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>baya</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>baya</t>
-        </is>
-      </c>
+          <t>kubeba</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>carry</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Italian</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>bacca</t>
+          <t>ढोना</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>bacca</t>
+          <t>ढोना</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -3180,168 +3251,923 @@
           <t>match</t>
         </is>
       </c>
+      <c r="F73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Welsh</t>
+          <t>Hungarian</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>aeron</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>aeronen</t>
-        </is>
-      </c>
+          <t>darál</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr">
         <is>
-          <t>match</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Japanese</t>
+          <t>Finnish</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ベリー</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>漿果</t>
-        </is>
-      </c>
+          <t>jauhaa</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Korean</t>
+          <t>Greek</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>말린 씨앗</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>장과</t>
-        </is>
-      </c>
+          <t>αλέθω</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Turkish</t>
+          <t>Russian</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>dut</t>
-        </is>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>tane</t>
-        </is>
-      </c>
+          <t>молоть</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>berry</t>
+          <t>grind</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Hebrew</t>
+          <t>German</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ברי</t>
-        </is>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>ענבה</t>
-        </is>
-      </c>
+          <t>schleifen</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>DIFFER</t>
-        </is>
-      </c>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>moler</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Italian</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>macinare</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Welsh</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>malu</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Vietnamese</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>xay</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>粉砕する</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Korean</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>갈기</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Thai</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>บด</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Indonesian</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>menggiling</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>öğütmek</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>طَحن</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Hebrew</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>לִטחוֹן</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Swahili</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>saga</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>grind</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Hindi</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>पिसना</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
           <t>berry</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Hungarian</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>bogyó</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>bogyó</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Finnish</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>marja</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>marja</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Greek</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>μούρο</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>ρόγα</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Russian</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ягода</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ягода</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>German</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Beere</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Beere</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Spanish</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>baya</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>baya</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Italian</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>bacca</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>bacca</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Welsh</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>aeron</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>aeronen</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>match</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Vietnamese</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>quả mọng</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Japanese</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>ベリー</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>漿果</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Korean</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>말린 씨앗</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>장과</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Thai</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>เบอร์รี่</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Indonesian</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>beri</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>dut</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>tane</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Arabic</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>بيري</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Hebrew</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ברי</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ענבה</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>DIFFER</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Swahili</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>beri</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>no-ref</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>berry</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
         <is>
           <t>Hindi</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>बेर</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>बेरी</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>match</t>
         </is>
       </c>
+      <c r="F109" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>